<commit_message>
added all effects in tech tree
</commit_message>
<xml_diff>
--- a/Tech tree.xlsx
+++ b/Tech tree.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gamin\Documents\Final year uni\Comp-3000\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\final year\Comp-3000\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CC0F593-1490-409B-BAB7-83583ADF5AD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FCEF087-1938-4E7B-9152-BCC93CF951DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aspects of game" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="178">
   <si>
     <t>Core aspects</t>
   </si>
@@ -529,6 +529,39 @@
   </si>
   <si>
     <t>Capacity is double and can now contain 2 resources not 1</t>
+  </si>
+  <si>
+    <t>Depot health is increased</t>
+  </si>
+  <si>
+    <t>Adds a sniper tower to the depot attacking nearby enemies</t>
+  </si>
+  <si>
+    <t>Adds a basic unit to the depot entrance to attack nearby enemies</t>
+  </si>
+  <si>
+    <t>Infilicts damage on zombies attacking the depot walls</t>
+  </si>
+  <si>
+    <t>Allows the player to buy minefields which explode on contact with zombie</t>
+  </si>
+  <si>
+    <t>Can now create Scout units</t>
+  </si>
+  <si>
+    <t>Can now create Sniper units</t>
+  </si>
+  <si>
+    <t>Can now create Melee units</t>
+  </si>
+  <si>
+    <t>Can now create Armoured Convoys</t>
+  </si>
+  <si>
+    <t>Can now create Medical Convoys</t>
+  </si>
+  <si>
+    <t>Can now create Fast Convoys</t>
   </si>
 </sst>
 </file>
@@ -662,12 +695,180 @@
   </cellStyles>
   <dxfs count="64">
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -684,174 +885,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -867,41 +900,41 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7936B949-188E-4582-8616-623FBF3C46A1}" name="Table1" displayName="Table1" ref="A1:D6" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7936B949-188E-4582-8616-623FBF3C46A1}" name="Table1" displayName="Table1" ref="A1:D6" totalsRowShown="0" headerRowDxfId="63" dataDxfId="62">
   <autoFilter ref="A1:D6" xr:uid="{7936B949-188E-4582-8616-623FBF3C46A1}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2EA6F07F-1C6E-40BA-AB5C-B295EB35CDCF}" name="Core aspects" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{194B2CAD-4A90-4E48-AEE8-DDC5F401A5C9}" name="Unit types" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{1448A4CC-616D-4E01-90A1-52101EAC6A7A}" name="Convoy types" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{B97AA103-9726-4AD2-A972-AE6976451B75}" name="Resources" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{2EA6F07F-1C6E-40BA-AB5C-B295EB35CDCF}" name="Core aspects" dataDxfId="61"/>
+    <tableColumn id="2" xr3:uid="{194B2CAD-4A90-4E48-AEE8-DDC5F401A5C9}" name="Unit types" dataDxfId="60"/>
+    <tableColumn id="3" xr3:uid="{1448A4CC-616D-4E01-90A1-52101EAC6A7A}" name="Convoy types" dataDxfId="59"/>
+    <tableColumn id="4" xr3:uid="{B97AA103-9726-4AD2-A972-AE6976451B75}" name="Resources" dataDxfId="58"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4B8BC961-7AD7-4C3B-AD78-4582E88561B3}" name="Table4" displayName="Table4" ref="A1:L9" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4B8BC961-7AD7-4C3B-AD78-4582E88561B3}" name="Table4" displayName="Table4" ref="A1:L9" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
   <autoFilter ref="A1:L9" xr:uid="{4B8BC961-7AD7-4C3B-AD78-4582E88561B3}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{273B543D-89B6-4955-A317-A6B9B4680CA3}" name="Defence upgrades" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{E2ECC974-9E12-4A07-BD63-BDCBEF1507C0}" name="Cost" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{2161316E-661A-4676-A677-BA66328341C0}" name="Pre-requsites" dataDxfId="17"/>
-    <tableColumn id="12" xr3:uid="{134C13E5-02FA-4F76-A06D-7102BADBA3D2}" name="Effect" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{CF1CB81C-0620-4735-BF49-5EF70D5A95D0}" name="Resource upgrades" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{D99D59BE-3DBC-4DC5-AC81-B6150EC1D1F4}" name="Cost2" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{02031DC9-8EF0-41F2-9B6C-598F6108A5A8}" name="Pre-requsites2" dataDxfId="14"/>
-    <tableColumn id="11" xr3:uid="{1680DD95-5CE0-4B9B-8549-ACF0137CB507}" name="Effect2" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{7E8E2876-1732-4CE0-B4F5-8E46B994DD1E}" name="Unit/Convoy unlocks" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{F2927B2C-24A0-4651-8D25-5F857B914BCE}" name="Cost3" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{DA739A9E-7639-4351-9932-0344E3EFE921}" name="Pre-requsites3" dataDxfId="10"/>
-    <tableColumn id="13" xr3:uid="{2CB92CE3-4985-4B3C-BB70-75B83BED998E}" name="Effect3" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{273B543D-89B6-4955-A317-A6B9B4680CA3}" name="Defence upgrades" dataDxfId="55"/>
+    <tableColumn id="5" xr3:uid="{E2ECC974-9E12-4A07-BD63-BDCBEF1507C0}" name="Cost" dataDxfId="54"/>
+    <tableColumn id="6" xr3:uid="{2161316E-661A-4676-A677-BA66328341C0}" name="Pre-requsites" dataDxfId="53"/>
+    <tableColumn id="12" xr3:uid="{134C13E5-02FA-4F76-A06D-7102BADBA3D2}" name="Effect" dataDxfId="52"/>
+    <tableColumn id="2" xr3:uid="{CF1CB81C-0620-4735-BF49-5EF70D5A95D0}" name="Resource upgrades" dataDxfId="51"/>
+    <tableColumn id="8" xr3:uid="{D99D59BE-3DBC-4DC5-AC81-B6150EC1D1F4}" name="Cost2" dataDxfId="50"/>
+    <tableColumn id="7" xr3:uid="{02031DC9-8EF0-41F2-9B6C-598F6108A5A8}" name="Pre-requsites2" dataDxfId="49"/>
+    <tableColumn id="11" xr3:uid="{1680DD95-5CE0-4B9B-8549-ACF0137CB507}" name="Effect2" dataDxfId="48"/>
+    <tableColumn id="3" xr3:uid="{7E8E2876-1732-4CE0-B4F5-8E46B994DD1E}" name="Unit/Convoy unlocks" dataDxfId="47"/>
+    <tableColumn id="9" xr3:uid="{F2927B2C-24A0-4651-8D25-5F857B914BCE}" name="Cost3" dataDxfId="46"/>
+    <tableColumn id="10" xr3:uid="{DA739A9E-7639-4351-9932-0344E3EFE921}" name="Pre-requsites3" dataDxfId="45"/>
+    <tableColumn id="13" xr3:uid="{2CB92CE3-4985-4B3C-BB70-75B83BED998E}" name="Effect3" dataDxfId="44"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A9CB1332-57FC-4281-A975-E180D5843E29}" name="Table2" displayName="Table2" ref="A1:T6" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A9CB1332-57FC-4281-A975-E180D5843E29}" name="Table2" displayName="Table2" ref="A1:T6" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
   <autoFilter ref="A1:T6" xr:uid="{A9CB1332-57FC-4281-A975-E180D5843E29}"/>
   <tableColumns count="20">
     <tableColumn id="2" xr3:uid="{E3DD0CDF-DC0D-4EB0-BEA2-5CE49EC8F866}" name="Generic upgrades" dataDxfId="41"/>
@@ -930,29 +963,29 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6F54F13A-D763-4415-AF52-3251B521332F}" name="Table24" displayName="Table24" ref="A1:T4" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6F54F13A-D763-4415-AF52-3251B521332F}" name="Table24" displayName="Table24" ref="A1:T4" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
   <autoFilter ref="A1:T4" xr:uid="{6F54F13A-D763-4415-AF52-3251B521332F}"/>
   <tableColumns count="20">
-    <tableColumn id="2" xr3:uid="{EB4E35EC-7A32-4043-AC4F-62F42A32D918}" name="Generic upgrades" dataDxfId="63"/>
-    <tableColumn id="3" xr3:uid="{B6D4A26B-841C-4651-B392-C413800BA49F}" name="Cost" dataDxfId="62"/>
-    <tableColumn id="5" xr3:uid="{92B340BF-E899-4C5E-A7EE-068FAE63D37E}" name="Pre-requisites" dataDxfId="61"/>
-    <tableColumn id="6" xr3:uid="{66255EC8-55E9-4791-B9A4-2658A7E89AB7}" name="Effect" dataDxfId="60"/>
-    <tableColumn id="7" xr3:uid="{8F1A242E-7826-4C78-A7FB-C0811E0DC38C}" name="Basic Convoy unique upgrades" dataDxfId="59"/>
-    <tableColumn id="8" xr3:uid="{880248A4-2E34-4E05-8EEE-19DAD8BA8D79}" name="Cost3" dataDxfId="58"/>
-    <tableColumn id="9" xr3:uid="{2AE87576-1799-432F-A7FD-846453B632F9}" name="Pre-requisites4" dataDxfId="57"/>
-    <tableColumn id="10" xr3:uid="{3D9BFB65-044E-46D6-BA79-605B541151F7}" name="Effect5" dataDxfId="56"/>
-    <tableColumn id="11" xr3:uid="{F2F0EDB8-2418-4120-A36E-6A799A139B44}" name="Armoured Convoy unique upgrades" dataDxfId="55"/>
-    <tableColumn id="12" xr3:uid="{74108871-80CF-4321-A45D-8AD943F641E5}" name="Cost4" dataDxfId="54"/>
-    <tableColumn id="13" xr3:uid="{528FAD47-5055-4C54-907C-AE802B24EE76}" name="Pre-requisites5" dataDxfId="53"/>
-    <tableColumn id="14" xr3:uid="{6FB45D9E-B476-4AAF-A885-1EE77EBB0A06}" name="Effect6" dataDxfId="52"/>
-    <tableColumn id="15" xr3:uid="{BA454E9F-DC7F-4486-A459-80E42B139783}" name="Medical Convoy unique upgrades" dataDxfId="51"/>
-    <tableColumn id="16" xr3:uid="{C32AC718-E815-45EA-97AD-9BBCB581C121}" name="Cost5" dataDxfId="50"/>
-    <tableColumn id="17" xr3:uid="{333DDDBD-0FA5-4B57-B26E-22C90DEAC453}" name="Pre-requisites6" dataDxfId="49"/>
-    <tableColumn id="18" xr3:uid="{DC44F460-C874-4BB4-946C-E222088CFB27}" name="Effect7" dataDxfId="48"/>
-    <tableColumn id="19" xr3:uid="{7EB0DD35-0EFD-4801-9E56-207D07409131}" name="Fast Convoy unique upgrades" dataDxfId="47"/>
-    <tableColumn id="20" xr3:uid="{242121C6-6B72-4769-BE45-504BC58B5446}" name="Cost6" dataDxfId="46"/>
-    <tableColumn id="21" xr3:uid="{1D20622B-A5D7-4451-BC95-05A11EC8C2F1}" name="Pre-requisites7" dataDxfId="45"/>
-    <tableColumn id="22" xr3:uid="{47D2D96E-45CA-4D18-9504-802D0C26A203}" name="Effect8" dataDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{EB4E35EC-7A32-4043-AC4F-62F42A32D918}" name="Generic upgrades" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{B6D4A26B-841C-4651-B392-C413800BA49F}" name="Cost" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{92B340BF-E899-4C5E-A7EE-068FAE63D37E}" name="Pre-requisites" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{66255EC8-55E9-4791-B9A4-2658A7E89AB7}" name="Effect" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{8F1A242E-7826-4C78-A7FB-C0811E0DC38C}" name="Basic Convoy unique upgrades" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{880248A4-2E34-4E05-8EEE-19DAD8BA8D79}" name="Cost3" dataDxfId="14"/>
+    <tableColumn id="9" xr3:uid="{2AE87576-1799-432F-A7FD-846453B632F9}" name="Pre-requisites4" dataDxfId="13"/>
+    <tableColumn id="10" xr3:uid="{3D9BFB65-044E-46D6-BA79-605B541151F7}" name="Effect5" dataDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{F2F0EDB8-2418-4120-A36E-6A799A139B44}" name="Armoured Convoy unique upgrades" dataDxfId="11"/>
+    <tableColumn id="12" xr3:uid="{74108871-80CF-4321-A45D-8AD943F641E5}" name="Cost4" dataDxfId="10"/>
+    <tableColumn id="13" xr3:uid="{528FAD47-5055-4C54-907C-AE802B24EE76}" name="Pre-requisites5" dataDxfId="9"/>
+    <tableColumn id="14" xr3:uid="{6FB45D9E-B476-4AAF-A885-1EE77EBB0A06}" name="Effect6" dataDxfId="8"/>
+    <tableColumn id="15" xr3:uid="{BA454E9F-DC7F-4486-A459-80E42B139783}" name="Medical Convoy unique upgrades" dataDxfId="7"/>
+    <tableColumn id="16" xr3:uid="{C32AC718-E815-45EA-97AD-9BBCB581C121}" name="Cost5" dataDxfId="6"/>
+    <tableColumn id="17" xr3:uid="{333DDDBD-0FA5-4B57-B26E-22C90DEAC453}" name="Pre-requisites6" dataDxfId="5"/>
+    <tableColumn id="18" xr3:uid="{DC44F460-C874-4BB4-946C-E222088CFB27}" name="Effect7" dataDxfId="4"/>
+    <tableColumn id="19" xr3:uid="{7EB0DD35-0EFD-4801-9E56-207D07409131}" name="Fast Convoy unique upgrades" dataDxfId="3"/>
+    <tableColumn id="20" xr3:uid="{242121C6-6B72-4769-BE45-504BC58B5446}" name="Cost6" dataDxfId="2"/>
+    <tableColumn id="21" xr3:uid="{1D20622B-A5D7-4451-BC95-05A11EC8C2F1}" name="Pre-requisites7" dataDxfId="1"/>
+    <tableColumn id="22" xr3:uid="{47D2D96E-45CA-4D18-9504-802D0C26A203}" name="Effect8" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1222,16 +1255,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" customWidth="1"/>
-    <col min="6" max="6" width="32.85546875" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" customWidth="1"/>
+    <col min="3" max="3" width="18.26953125" customWidth="1"/>
+    <col min="4" max="4" width="14.453125" customWidth="1"/>
+    <col min="6" max="6" width="32.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1248,7 +1281,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -1265,7 +1298,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
@@ -1279,7 +1312,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
@@ -1293,7 +1326,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1307,7 +1340,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -1326,23 +1359,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7C1AE8C-0057-4B1D-8955-2B721776BB0B}">
   <dimension ref="A1:L9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="3" width="21.28515625" customWidth="1"/>
-    <col min="4" max="4" width="28.140625" customWidth="1"/>
-    <col min="5" max="5" width="27.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.1796875" customWidth="1"/>
+    <col min="2" max="2" width="22.7265625" customWidth="1"/>
+    <col min="3" max="3" width="21.26953125" customWidth="1"/>
+    <col min="4" max="4" width="28.1796875" customWidth="1"/>
+    <col min="5" max="5" width="27.81640625" customWidth="1"/>
     <col min="6" max="6" width="19" customWidth="1"/>
-    <col min="7" max="7" width="27.85546875" customWidth="1"/>
-    <col min="8" max="8" width="28.28515625" customWidth="1"/>
-    <col min="9" max="9" width="25.28515625" customWidth="1"/>
-    <col min="10" max="10" width="26.28515625" customWidth="1"/>
-    <col min="11" max="11" width="28.28515625" customWidth="1"/>
-    <col min="12" max="12" width="15.140625" customWidth="1"/>
+    <col min="7" max="7" width="27.81640625" customWidth="1"/>
+    <col min="8" max="8" width="28.26953125" customWidth="1"/>
+    <col min="9" max="9" width="25.26953125" customWidth="1"/>
+    <col min="10" max="10" width="26.26953125" customWidth="1"/>
+    <col min="11" max="11" width="28.26953125" customWidth="1"/>
+    <col min="12" max="12" width="15.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>24</v>
       </c>
@@ -1380,7 +1413,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>38</v>
       </c>
@@ -1388,7 +1421,9 @@
       <c r="C2" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="9"/>
+      <c r="D2" s="9" t="s">
+        <v>167</v>
+      </c>
       <c r="E2" s="8" t="s">
         <v>46</v>
       </c>
@@ -1406,9 +1441,11 @@
       <c r="K2" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="L2" s="3"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L2" s="3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
         <v>39</v>
       </c>
@@ -1416,7 +1453,9 @@
       <c r="C3" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="8"/>
+      <c r="D3" s="6" t="s">
+        <v>168</v>
+      </c>
       <c r="E3" s="8" t="s">
         <v>47</v>
       </c>
@@ -1434,9 +1473,11 @@
       <c r="K3" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="L3" s="3"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L3" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>42</v>
       </c>
@@ -1444,7 +1485,9 @@
       <c r="C4" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D4" s="3"/>
+      <c r="D4" s="7" t="s">
+        <v>169</v>
+      </c>
       <c r="E4" s="8" t="s">
         <v>48</v>
       </c>
@@ -1462,9 +1505,11 @@
       <c r="K4" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="L4" s="3"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L4" s="7" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>43</v>
       </c>
@@ -1472,7 +1517,9 @@
       <c r="C5" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D5" s="3"/>
+      <c r="D5" s="7" t="s">
+        <v>170</v>
+      </c>
       <c r="E5" s="8" t="s">
         <v>65</v>
       </c>
@@ -1490,9 +1537,11 @@
       <c r="K5" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="L5" s="3"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L5" s="7" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>45</v>
       </c>
@@ -1500,7 +1549,9 @@
       <c r="C6" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="3"/>
+      <c r="D6" s="7" t="s">
+        <v>171</v>
+      </c>
       <c r="E6" s="3" t="s">
         <v>49</v>
       </c>
@@ -1518,9 +1569,11 @@
       <c r="K6" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="L6" s="3"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L6" s="7" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -1542,9 +1595,11 @@
       <c r="K7" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="L7" s="3"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L7" s="7" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -1564,7 +1619,7 @@
       <c r="K8" s="3"/>
       <c r="L8" s="3"/>
     </row>
-    <row r="9" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -1594,31 +1649,31 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAF4865F-6BB8-4976-9DE5-36DB3EE7176D}">
   <dimension ref="A1:T6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" customWidth="1"/>
-    <col min="2" max="2" width="31.7109375" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" customWidth="1"/>
-    <col min="4" max="4" width="24.140625" customWidth="1"/>
+    <col min="1" max="1" width="20.7265625" customWidth="1"/>
+    <col min="2" max="2" width="31.7265625" customWidth="1"/>
+    <col min="3" max="3" width="19.1796875" customWidth="1"/>
+    <col min="4" max="4" width="24.1796875" customWidth="1"/>
     <col min="5" max="5" width="31" customWidth="1"/>
-    <col min="6" max="6" width="19.7109375" customWidth="1"/>
-    <col min="7" max="7" width="25.140625" customWidth="1"/>
-    <col min="8" max="8" width="30.28515625" customWidth="1"/>
-    <col min="9" max="9" width="21.7109375" customWidth="1"/>
-    <col min="10" max="10" width="37.7109375" customWidth="1"/>
-    <col min="11" max="11" width="27.140625" customWidth="1"/>
-    <col min="12" max="12" width="30.7109375" customWidth="1"/>
-    <col min="13" max="13" width="27.5703125" customWidth="1"/>
-    <col min="14" max="14" width="27.42578125" customWidth="1"/>
-    <col min="15" max="15" width="24.28515625" customWidth="1"/>
-    <col min="16" max="16" width="34.7109375" customWidth="1"/>
-    <col min="17" max="17" width="21.140625" customWidth="1"/>
-    <col min="18" max="18" width="33.140625" customWidth="1"/>
-    <col min="19" max="19" width="34.140625" customWidth="1"/>
-    <col min="20" max="20" width="32.28515625" customWidth="1"/>
+    <col min="6" max="6" width="19.7265625" customWidth="1"/>
+    <col min="7" max="7" width="25.1796875" customWidth="1"/>
+    <col min="8" max="8" width="30.26953125" customWidth="1"/>
+    <col min="9" max="9" width="21.7265625" customWidth="1"/>
+    <col min="10" max="10" width="37.7265625" customWidth="1"/>
+    <col min="11" max="11" width="27.1796875" customWidth="1"/>
+    <col min="12" max="12" width="30.7265625" customWidth="1"/>
+    <col min="13" max="13" width="27.54296875" customWidth="1"/>
+    <col min="14" max="14" width="27.453125" customWidth="1"/>
+    <col min="15" max="15" width="24.26953125" customWidth="1"/>
+    <col min="16" max="16" width="34.7265625" customWidth="1"/>
+    <col min="17" max="17" width="21.1796875" customWidth="1"/>
+    <col min="18" max="18" width="33.1796875" customWidth="1"/>
+    <col min="19" max="19" width="34.1796875" customWidth="1"/>
+    <col min="20" max="20" width="32.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>19</v>
       </c>
@@ -1680,7 +1735,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
         <v>79</v>
       </c>
@@ -1736,7 +1791,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="3" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
         <v>80</v>
       </c>
@@ -1792,7 +1847,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>81</v>
       </c>
@@ -1848,7 +1903,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="5" spans="1:20" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" ht="39" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -1890,7 +1945,7 @@
       <c r="S5" s="3"/>
       <c r="T5" s="3"/>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -1931,31 +1986,31 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73FA7BAE-C73F-432A-B85B-06103167559F}">
   <dimension ref="A1:T4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" customWidth="1"/>
-    <col min="2" max="2" width="35.85546875" customWidth="1"/>
-    <col min="3" max="3" width="34.28515625" customWidth="1"/>
+    <col min="1" max="1" width="19.7265625" customWidth="1"/>
+    <col min="2" max="2" width="35.81640625" customWidth="1"/>
+    <col min="3" max="3" width="34.26953125" customWidth="1"/>
     <col min="4" max="4" width="37" customWidth="1"/>
-    <col min="5" max="5" width="30.5703125" customWidth="1"/>
-    <col min="6" max="6" width="31.140625" customWidth="1"/>
-    <col min="7" max="7" width="30.5703125" customWidth="1"/>
-    <col min="8" max="8" width="32.85546875" customWidth="1"/>
-    <col min="9" max="9" width="34.140625" customWidth="1"/>
-    <col min="10" max="10" width="31.140625" customWidth="1"/>
-    <col min="11" max="11" width="30.28515625" customWidth="1"/>
-    <col min="12" max="12" width="39.28515625" customWidth="1"/>
-    <col min="13" max="13" width="32.7109375" customWidth="1"/>
-    <col min="14" max="14" width="36.28515625" customWidth="1"/>
-    <col min="15" max="15" width="50.28515625" customWidth="1"/>
-    <col min="16" max="16" width="38.28515625" customWidth="1"/>
-    <col min="17" max="17" width="29.7109375" customWidth="1"/>
-    <col min="18" max="18" width="23.5703125" customWidth="1"/>
-    <col min="19" max="19" width="25.42578125" customWidth="1"/>
+    <col min="5" max="5" width="30.54296875" customWidth="1"/>
+    <col min="6" max="6" width="31.1796875" customWidth="1"/>
+    <col min="7" max="7" width="30.54296875" customWidth="1"/>
+    <col min="8" max="8" width="32.81640625" customWidth="1"/>
+    <col min="9" max="9" width="34.1796875" customWidth="1"/>
+    <col min="10" max="10" width="31.1796875" customWidth="1"/>
+    <col min="11" max="11" width="30.26953125" customWidth="1"/>
+    <col min="12" max="12" width="39.26953125" customWidth="1"/>
+    <col min="13" max="13" width="32.7265625" customWidth="1"/>
+    <col min="14" max="14" width="36.26953125" customWidth="1"/>
+    <col min="15" max="15" width="50.26953125" customWidth="1"/>
+    <col min="16" max="16" width="38.26953125" customWidth="1"/>
+    <col min="17" max="17" width="29.7265625" customWidth="1"/>
+    <col min="18" max="18" width="23.54296875" customWidth="1"/>
+    <col min="19" max="19" width="25.453125" customWidth="1"/>
     <col min="20" max="20" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>19</v>
       </c>
@@ -2017,7 +2072,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>96</v>
       </c>
@@ -2069,7 +2124,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="3" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>97</v>
       </c>
@@ -2121,7 +2176,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="60" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="7"/>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>

</xml_diff>